<commit_message>
Tambah jenjang (SD/SMP/SMA/SMK) pada template & bank soal + cache-busting v2 + file contoh soal baru
- template-soal.docx: baris JENJANG di bawah KODE SOAL (parser deteksi & sebarkan ke semua soal dalam paket)
- docx-parser.js: deteksi JENJANG -> s.jenjang
- schema.sql: kolom jenjang di soal_bank + RPC bank_soal/simpan_soal
- guru.html: badge jenjang, dropdown edit, filter & pencarian jenjang, payload upload
- seed.sql & mock api.js: jenjang di data demo
- admin/index/guru.html: cache-busting ?v=2 untuk css/js
- template: contoh soal TKA Bahasa Indonesia SD + template siswa diperbarui
</commit_message>
<xml_diff>
--- a/template/template-siswa.xlsx
+++ b/template/template-siswa.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
   <si>
     <t xml:space="preserve">NIS</t>
   </si>
@@ -46,46 +46,52 @@
     <t xml:space="preserve">XII IPA 1</t>
   </si>
   <si>
-    <t xml:space="preserve">ani</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ani123</t>
+    <t xml:space="preserve">budi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">budi123</t>
   </si>
   <si>
     <t xml:space="preserve">2026002</t>
   </si>
   <si>
-    <t xml:space="preserve">Siti Rahayu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anis123</t>
+    <t xml:space="preserve">Ratna Sri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ratna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ratna123</t>
   </si>
   <si>
     <t xml:space="preserve">2026003</t>
   </si>
   <si>
+    <t xml:space="preserve">Monika</t>
+  </si>
+  <si>
     <t xml:space="preserve">XII IPA 2</t>
   </si>
   <si>
-    <t xml:space="preserve">anisa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anisa123</t>
+    <t xml:space="preserve">monika</t>
+  </si>
+  <si>
+    <t xml:space="preserve">monika123</t>
   </si>
   <si>
     <t xml:space="preserve">2026004</t>
   </si>
   <si>
+    <t xml:space="preserve">Roycoo</t>
+  </si>
+  <si>
     <t xml:space="preserve">XII IPA 3</t>
   </si>
   <si>
-    <t xml:space="preserve">anisah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">anisah123</t>
+    <t xml:space="preserve">roycoo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">roycoo123</t>
   </si>
 </sst>
 </file>
@@ -421,34 +427,34 @@
         <v>14</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F5" s="1"/>
     </row>

</xml_diff>

<commit_message>
Implement generate kartu siswa fitur print PDF A4 (6-8 kartu/halaman)
</commit_message>
<xml_diff>
--- a/template/template-siswa.xlsx
+++ b/template/template-siswa.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t xml:space="preserve">NIS</t>
   </si>
@@ -34,9 +34,6 @@
     <t xml:space="preserve">Username</t>
   </si>
   <si>
-    <t xml:space="preserve">Password</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026001</t>
   </si>
   <si>
@@ -46,24 +43,12 @@
     <t xml:space="preserve">XII IPA 1</t>
   </si>
   <si>
-    <t xml:space="preserve">budi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">budi123</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026002</t>
   </si>
   <si>
     <t xml:space="preserve">Ratna Sri</t>
   </si>
   <si>
-    <t xml:space="preserve">ratna</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ratna123</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026003</t>
   </si>
   <si>
@@ -73,12 +58,6 @@
     <t xml:space="preserve">XII IPA 2</t>
   </si>
   <si>
-    <t xml:space="preserve">monika</t>
-  </si>
-  <si>
-    <t xml:space="preserve">monika123</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026004</t>
   </si>
   <si>
@@ -86,12 +65,6 @@
   </si>
   <si>
     <t xml:space="preserve">XII IPA 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">roycoo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">roycoo123</t>
   </si>
 </sst>
 </file>
@@ -365,8 +338,11 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
-  <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="9.34"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -381,82 +357,71 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1"/>
+      <c r="E1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="1"/>
+      <c r="D2" s="1" t="str">
+        <f aca="false">A2</f>
+        <v>2026001</v>
+      </c>
+      <c r="E2" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="1"/>
+        <v>6</v>
+      </c>
+      <c r="D3" s="1" t="str">
+        <f aca="false">A3</f>
+        <v>2026002</v>
+      </c>
+      <c r="E3" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F4" s="1"/>
+        <v>11</v>
+      </c>
+      <c r="D4" s="1" t="str">
+        <f aca="false">A4</f>
+        <v>2026003</v>
+      </c>
+      <c r="E4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" s="1"/>
+        <v>14</v>
+      </c>
+      <c r="D5" s="1" t="str">
+        <f aca="false">A5</f>
+        <v>2026004</v>
+      </c>
+      <c r="E5" s="1"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
Perbarui template import siswa ke kolom NIS/Nama/Kelas/Username + teks panduan impor
</commit_message>
<xml_diff>
--- a/template/template-siswa.xlsx
+++ b/template/template-siswa.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t xml:space="preserve">NIS</t>
   </si>
@@ -34,37 +34,49 @@
     <t xml:space="preserve">Username</t>
   </si>
   <si>
-    <t xml:space="preserve">2026001</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budi Santoso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XII IPA 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026002</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ratna Sri</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026003</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monika</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XII IPA 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026004</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Roycoo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">XII IPA 3</t>
+    <t xml:space="preserve">Andi Susanto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X MIPA 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budi Raharjo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Citra Lestari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X MIPA 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dewi Maharani</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Eko Prasetyo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">X IPS 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fajar Sidiq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gita Savitri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XI MIPA 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hadi Pranoto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intan Nuraini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XI IPS 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Joko Widodo</t>
   </si>
 </sst>
 </file>
@@ -140,12 +152,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -338,90 +358,171 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.50390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="9.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="1" width="9.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1"/>
+      <c r="E1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="n">
+        <v>260001</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="3" t="n">
+        <v>260001</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="n">
+        <v>260002</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="str">
-        <f aca="false">A2</f>
-        <v>2026001</v>
-      </c>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="C3" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>260002</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="n">
+        <v>260003</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" s="1" t="str">
-        <f aca="false">A3</f>
-        <v>2026002</v>
-      </c>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="D4" s="3" t="n">
+        <v>260003</v>
+      </c>
+      <c r="E4" s="2"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="n">
+        <v>260004</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>260004</v>
+      </c>
+      <c r="E5" s="2"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="n">
+        <v>260005</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="1" t="str">
-        <f aca="false">A4</f>
-        <v>2026003</v>
-      </c>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="D6" s="3" t="n">
+        <v>260005</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="n">
+        <v>260006</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="C7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>260006</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="n">
+        <v>260007</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="1" t="str">
-        <f aca="false">A5</f>
-        <v>2026004</v>
-      </c>
-      <c r="E5" s="1"/>
+      <c r="D8" s="3" t="n">
+        <v>260007</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="n">
+        <v>260008</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>260008</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="n">
+        <v>260009</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>260009</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="n">
+        <v>260010</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>260010</v>
+      </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>